<commit_message>
Refine attachment packaging and CLID exports
</commit_message>
<xml_diff>
--- a/backend/data/templates/clid-item-template.xlsx
+++ b/backend/data/templates/clid-item-template.xlsx
@@ -1,21 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\pacote_teste\Documentos CLID\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03EF91C-CE28-4591-8D35-C6642E16DDC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Contract Header" r:id="rId3" sheetId="1"/>
-    <sheet name="Contract Item Information" r:id="rId4" sheetId="2"/>
-    <sheet name="Header Attributes" r:id="rId5" sheetId="3"/>
-    <sheet name="Item Attributes" r:id="rId6" sheetId="4"/>
+    <sheet name="Contract Header" sheetId="1" r:id="rId1"/>
+    <sheet name="Contract Item Information" sheetId="2" r:id="rId2"/>
+    <sheet name="Header Attributes" sheetId="3" r:id="rId3"/>
+    <sheet name="Item Attributes" sheetId="4" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="103">
   <si>
     <t/>
   </si>
@@ -221,9 +229,6 @@
   </si>
   <si>
     <t>0000000001</t>
-  </si>
-  <si>
-    <t>12</t>
   </si>
   <si>
     <t>Attribute Name</t>
@@ -334,21 +339,21 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="12"/>
       <name val="Calibri"/>
-      <sz val="11.0"/>
-      <color indexed="12"/>
-      <b val="true"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -356,74 +361,27 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="darkGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="31"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="31"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <top style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin"/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -438,59 +396,371 @@
       <bottom style="thin">
         <color indexed="8"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyAlignment="true" applyFont="true" applyFill="true" applyBorder="true">
-      <alignment wrapText="true" horizontal="left" vertical="top"/>
-      <protection locked="true"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
-      <alignment wrapText="true" horizontal="left" vertical="top"/>
-      <protection locked="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
-      <alignment wrapText="true" horizontal="left" vertical="top"/>
-      <protection locked="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <outlinePr summaryBelow="false" summaryRight="false"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:S6"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.0" customWidth="true"/>
-    <col min="2" max="2" width="15.0" customWidth="true"/>
-    <col min="3" max="3" width="15.0" customWidth="true"/>
-    <col min="4" max="4" width="15.0" customWidth="true"/>
-    <col min="5" max="5" width="15.0" customWidth="true"/>
-    <col min="6" max="6" width="15.0" customWidth="true"/>
-    <col min="7" max="7" width="15.0" customWidth="true"/>
-    <col min="8" max="8" width="15.0" customWidth="true"/>
-    <col min="9" max="9" width="15.0" customWidth="true"/>
-    <col min="10" max="10" width="15.0" customWidth="true"/>
-    <col min="11" max="11" width="15.0" customWidth="true"/>
-    <col min="12" max="12" width="15.0" customWidth="true"/>
-    <col min="13" max="13" width="15.0" customWidth="true"/>
-    <col min="14" max="14" width="15.0" customWidth="true"/>
-    <col min="15" max="15" width="15.0" customWidth="true"/>
-    <col min="16" max="16" width="15.0" customWidth="true"/>
-    <col min="17" max="17" width="15.0" customWidth="true"/>
-    <col min="18" max="18" width="15.0" customWidth="true"/>
-    <col min="19" max="19" width="15.0" customWidth="true"/>
+    <col min="1" max="19" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -549,7 +819,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
@@ -586,7 +856,7 @@
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -611,7 +881,7 @@
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -636,7 +906,7 @@
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -661,7 +931,7 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -687,48 +957,24 @@
       <c r="S6" s="2"/>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
-    <outlinePr summaryBelow="false" summaryRight="false"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AA2"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.0" customWidth="true"/>
-    <col min="2" max="2" width="15.0" customWidth="true"/>
-    <col min="3" max="3" width="15.0" customWidth="true"/>
-    <col min="4" max="4" width="15.0" customWidth="true"/>
-    <col min="5" max="5" width="15.0" customWidth="true"/>
-    <col min="6" max="6" width="15.0" customWidth="true"/>
-    <col min="7" max="7" width="15.0" customWidth="true"/>
-    <col min="8" max="8" width="15.0" customWidth="true"/>
-    <col min="9" max="9" width="15.0" customWidth="true"/>
-    <col min="10" max="10" width="15.0" customWidth="true"/>
-    <col min="11" max="11" width="15.0" customWidth="true"/>
-    <col min="12" max="12" width="15.0" customWidth="true"/>
-    <col min="13" max="13" width="15.0" customWidth="true"/>
-    <col min="14" max="14" width="15.0" customWidth="true"/>
-    <col min="15" max="15" width="15.0" customWidth="true"/>
-    <col min="16" max="16" width="15.0" customWidth="true"/>
-    <col min="17" max="17" width="15.0" customWidth="true"/>
-    <col min="18" max="18" width="15.0" customWidth="true"/>
-    <col min="19" max="19" width="15.0" customWidth="true"/>
-    <col min="20" max="20" width="15.0" customWidth="true"/>
-    <col min="21" max="21" width="15.0" customWidth="true"/>
-    <col min="22" max="22" width="10.0" customWidth="true"/>
-    <col min="23" max="23" width="15.0" customWidth="true"/>
-    <col min="24" max="24" width="15.0" customWidth="true"/>
-    <col min="25" max="25" width="15.0" customWidth="true"/>
-    <col min="26" max="26" width="15.0" customWidth="true"/>
-    <col min="27" max="27" width="15.0" customWidth="true"/>
+    <col min="1" max="21" width="15" customWidth="1"/>
+    <col min="22" max="22" width="10" customWidth="1"/>
+    <col min="23" max="27" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:27" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
@@ -811,7 +1057,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:27" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>58</v>
@@ -825,7 +1071,9 @@
       <c r="E2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="G2" s="2" t="s">
         <v>61</v>
       </c>
@@ -853,239 +1101,230 @@
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
+      <c r="V2" s="4">
+        <v>10</v>
+      </c>
       <c r="W2" s="2" t="s">
         <v>67</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="Y2" s="2" t="s">
-        <v>68</v>
+      <c r="Y2" s="2">
+        <v>10</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
-    <outlinePr summaryBelow="false" summaryRight="false"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.0" customWidth="true"/>
-    <col min="2" max="2" width="15.0" customWidth="true"/>
-    <col min="3" max="3" width="15.0" customWidth="true"/>
-    <col min="4" max="4" width="15.0" customWidth="true"/>
-    <col min="5" max="5" width="15.0" customWidth="true"/>
-    <col min="6" max="6" width="15.0" customWidth="true"/>
+    <col min="1" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
-    <outlinePr summaryBelow="false" summaryRight="false"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:I15"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.0" customWidth="true"/>
-    <col min="2" max="2" width="15.0" customWidth="true"/>
-    <col min="3" max="3" width="15.0" customWidth="true"/>
-    <col min="4" max="4" width="15.0" customWidth="true"/>
-    <col min="5" max="5" width="15.0" customWidth="true"/>
-    <col min="6" max="6" width="15.0" customWidth="true"/>
-    <col min="7" max="7" width="15.0" customWidth="true"/>
-    <col min="8" max="8" width="15.0" customWidth="true"/>
-    <col min="9" max="9" width="15.0" customWidth="true"/>
+    <col min="1" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="34.42578125" customWidth="1"/>
+    <col min="7" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="2">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>58</v>
       </c>
@@ -1093,24 +1332,24 @@
         <v>53</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>53</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>58</v>
       </c>
@@ -1118,199 +1357,199 @@
         <v>42</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>42</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>